<commit_message>
Demo app.py để chạy thử và đánh giá mô hình (đã loại bỏ file pkl nặng)
</commit_message>
<xml_diff>
--- a/notebooks/Model_Comparison/results/model_comparison/cv_metrics.xlsx
+++ b/notebooks/Model_Comparison/results/model_comparison/cv_metrics.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,17 +417,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Mean CV MAE</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Std CV MAE</t>
         </is>
@@ -448,27 +436,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Random Forest</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>25370.04751593934</v>
+        <v>3840.266298299042</v>
       </c>
       <c r="C2" t="n">
-        <v>6175.444957811656</v>
+        <v>72.98940774155628</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>Random Forest</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>25434.26970741986</v>
+        <v>3863.056351290154</v>
       </c>
       <c r="C3" t="n">
-        <v>6244.522956169497</v>
+        <v>60.42352160648753</v>
       </c>
     </row>
     <row r="4">
@@ -478,10 +466,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>25785.06124072428</v>
+        <v>3923.357494612707</v>
       </c>
       <c r="C4" t="n">
-        <v>6264.463860468543</v>
+        <v>81.62061174673474</v>
       </c>
     </row>
     <row r="5">
@@ -491,62 +479,62 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>26829.73645404756</v>
+        <v>4308.052125324122</v>
       </c>
       <c r="C5" t="n">
-        <v>6301.767940801004</v>
+        <v>92.5349219198899</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Linear Regression</t>
+          <t>Dummy Regressor</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>28962.26005037715</v>
+        <v>6356.655887811791</v>
       </c>
       <c r="C6" t="n">
-        <v>6416.356398921576</v>
+        <v>115.174950841938</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Ridge</t>
+          <t>Linear Regression</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>28962.83705544929</v>
+        <v>2328369.846633664</v>
       </c>
       <c r="C7" t="n">
-        <v>6415.860840906339</v>
+        <v>4646149.877287298</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Lasso</t>
+          <t>Ridge</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>30838.67917495368</v>
+        <v>2328369.88564757</v>
       </c>
       <c r="C8" t="n">
-        <v>6332.302528408619</v>
+        <v>4646150.13781618</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Dummy Regressor</t>
+          <t>Lasso</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>30838.67917495368</v>
+        <v>2329470.392880273</v>
       </c>
       <c r="C9" t="n">
-        <v>6332.302528408619</v>
+        <v>4646149.086262577</v>
       </c>
     </row>
   </sheetData>

</xml_diff>